<commit_message>
changed section order in jupyter book, updated imports
</commit_message>
<xml_diff>
--- a/EIANN/data/supplementary_tables/Table_S6_mnist_hyperparams_part1.xlsx
+++ b/EIANN/data/supplementary_tables/Table_S6_mnist_hyperparams_part1.xlsx
@@ -478,7 +478,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Winit (H1)</t>
+          <t>W_init (H1)</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -542,7 +542,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Winit (H2)</t>
+          <t>W_init (H2)</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -606,7 +606,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Winit (Output)</t>
+          <t>W_init (Output)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -662,7 +662,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Yinit (SomaI, H1)</t>
+          <t>Y_init (SomaI, H1)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -700,7 +700,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Winit (SomaI, H1)</t>
+          <t>W_init (SomaI, H1)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -738,7 +738,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Qinit (SomaI, H1)</t>
+          <t>Q_init (SomaI, H1)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -776,7 +776,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rinit (SomaI, H1)</t>
+          <t>R_init (SomaI, H1)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -814,7 +814,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Yinit (SomaI, H2)</t>
+          <t>Y_init (SomaI, H2)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -852,7 +852,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Winit (SomaI, H2)</t>
+          <t>W_init (SomaI, H2)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -890,7 +890,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Qinit (SomaI, H2)</t>
+          <t>Q_init (SomaI, H2)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -928,7 +928,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Rinit (SomaI, H2)</t>
+          <t>R_init (SomaI, H2)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -966,7 +966,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Yinit (SomaI, Output)</t>
+          <t>Y_init (SomaI, Output)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1004,7 +1004,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Winit (SomaI, Output)</t>
+          <t>W_init (SomaI, Output)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1042,7 +1042,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Qinit (SomaI, Output)</t>
+          <t>Q_init (SomaI, Output)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1080,7 +1080,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Rinit (SomaI, Output)</t>
+          <t>R_init (SomaI, Output)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1574,7 +1574,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Wsum (H1)</t>
+          <t>W_sum (H1)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1614,7 +1614,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Ysum (SomaI, H1)</t>
+          <t>Y_sum (SomaI, H1)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1654,7 +1654,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Wsum (SomaI, H1)</t>
+          <t>W_sum (SomaI, H1)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1694,7 +1694,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Qsum (SomaI, H1)</t>
+          <t>Q_sum (SomaI, H1)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1734,7 +1734,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Rsum (SomaI, H1)</t>
+          <t>R_sum (SomaI, H1)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1774,7 +1774,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Wsum (H2)</t>
+          <t>W_sum (H2)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1814,7 +1814,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Ysum (SomaI, H2)</t>
+          <t>Y_sum (SomaI, H2)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1854,7 +1854,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Wsum (SomaI, H2)</t>
+          <t>W_sum (SomaI, H2)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1894,7 +1894,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Qsum (SomaI, H2)</t>
+          <t>Q_sum (SomaI, H2)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1934,7 +1934,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Rsum (SomaI, H2)</t>
+          <t>R_sum (SomaI, H2)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1974,7 +1974,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ysum (SomaI, Output)</t>
+          <t>Y_sum (SomaI, Output)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2014,7 +2014,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Wsum (SomaI, Output)</t>
+          <t>W_sum (SomaI, Output)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2054,7 +2054,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Qsum (SomaI, Output)</t>
+          <t>Q_sum (SomaI, Output)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2094,7 +2094,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Rsum (SomaI, Output)</t>
+          <t>R_sum (SomaI, Output)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">

</xml_diff>